<commit_message>
feat: add healing potion items
</commit_message>
<xml_diff>
--- a/DataTable/ItemDataTable.xlsx
+++ b/DataTable/ItemDataTable.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ItemTable(재민)" sheetId="1" r:id="Rf4ba63e715314433"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ItemGroupTable(밸런스x, 컨셉 위주 작성)" sheetId="2" r:id="R7ca049668cda4ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ItemTable(재민)" sheetId="1" r:id="Re5b945cefffa4e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ItemGroupTable(밸런스x, 컨셉 위주 작성)" sheetId="2" r:id="R60f5231915aa44a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1624,30 +1624,70 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1"/>
-      <x:c r="B24" s="30"/>
-      <x:c r="C24" s="31"/>
-      <x:c r="D24" s="32"/>
-      <x:c r="E24" s="33"/>
-      <x:c r="F24" s="33"/>
-      <x:c r="G24" s="33"/>
-      <x:c r="H24" s="33"/>
-      <x:c r="I24" s="37"/>
-      <x:c r="J24" s="30"/>
-      <x:c r="K24" s="35"/>
+      <x:c r="B24" s="30" t="str">
+        <x:v>개인 회복약</x:v>
+      </x:c>
+      <x:c r="C24" s="31" t="str">
+        <x:v>personal_healing_potion</x:v>
+      </x:c>
+      <x:c r="D24" s="32" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E24" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F24" s="33" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G24" s="33" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H24" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="37" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="J24" s="30" t="str">
+        <x:v>개인 회복약</x:v>
+      </x:c>
+      <x:c r="K24" s="35" t="str">
+        <x:v>아군 한 명의 체력이 50% 미만이 되면 자동으로 사용해 해당 아군의 최대 체력의 {0}%를 회복한다. 최대 {1}개까지 보유할 수 있다.</x:v>
+      </x:c>
       <x:c r="L24" s="36"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1"/>
-      <x:c r="B25" s="30"/>
-      <x:c r="C25" s="31"/>
-      <x:c r="D25" s="32"/>
-      <x:c r="E25" s="33"/>
-      <x:c r="F25" s="33"/>
-      <x:c r="G25" s="33"/>
-      <x:c r="H25" s="33"/>
-      <x:c r="I25" s="37"/>
-      <x:c r="J25" s="30"/>
-      <x:c r="K25" s="35"/>
+      <x:c r="B25" s="30" t="str">
+        <x:v>단체 회복약</x:v>
+      </x:c>
+      <x:c r="C25" s="31" t="str">
+        <x:v>party_healing_potion</x:v>
+      </x:c>
+      <x:c r="D25" s="32" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E25" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F25" s="33" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="G25" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H25" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="37" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="J25" s="30" t="str">
+        <x:v>단체 회복약</x:v>
+      </x:c>
+      <x:c r="K25" s="35" t="str">
+        <x:v>아군 한 명의 체력이 50% 미만이 되면 자동으로 사용해 살아 있는 모든 아군의 최대 체력의 {0}%를 회복한다. 최대 {1}개까지 보유할 수 있다.</x:v>
+      </x:c>
       <x:c r="L25" s="36"/>
     </x:row>
     <x:row r="26">

</xml_diff>